<commit_message>
update cum 1 thanh xoan
</commit_message>
<xml_diff>
--- a/Documents/params_plant.xlsx
+++ b/Documents/params_plant.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f8b1db9dde50c834/Desktop/git/Adaptive-EPS-using-Reinforcement-Learning/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B38EDF5-F506-40DC-BB8F-60A503B1E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{4B38EDF5-F506-40DC-BB8F-60A503B1E908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE9B0956-83FA-49F6-86F2-AD0480918186}"/>
   <bookViews>
-    <workbookView xWindow="1104" yWindow="2976" windowWidth="23040" windowHeight="12120" xr2:uid="{C5D89282-197A-4397-95BA-6EB3964BEC76}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{C5D89282-197A-4397-95BA-6EB3964BEC76}"/>
   </bookViews>
   <sheets>
     <sheet name="Cum1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="67">
   <si>
     <t>ten_dai_luong</t>
   </si>
@@ -58,54 +58,21 @@
     <t>nguon</t>
   </si>
   <si>
-    <t>J_total</t>
-  </si>
-  <si>
     <t>kg.m^2</t>
   </si>
   <si>
-    <t>Tổng quán tính quy đổi về trục theta của toàn bộ cơ cấu lái (vô-lăng + cột lái + rotor motor trợ lực qua tỷ số truyền + thanh răng qua pinion + 2 bánh trước qua king-pin)</t>
-  </si>
-  <si>
-    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, PT(14): J_total = J1+J2 = 0.044+0.11, đo thực nghiệm trên xe Hyundai i30 bằng nhận dạng hệ thống (system identification)</t>
-  </si>
-  <si>
-    <t>B_total</t>
-  </si>
-  <si>
     <t>N.m.s/rad</t>
   </si>
   <si>
-    <t>Tổng hệ số ma sát nhớt quy đổi về trục theta (cột lái + rotor motor qua tỷ số truyền + thanh răng qua pinion)</t>
-  </si>
-  <si>
-    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, PT(14): B_total = C1+C2 = 0.25+1.35, cùng phép đo với J_total</t>
-  </si>
-  <si>
-    <t>T_f_total</t>
-  </si>
-  <si>
     <t>N.m</t>
   </si>
   <si>
-    <t>Mô-men ma sát khô Coulomb quy đổi về trục theta (ma sát bánh răng motor-cột lái và thước lái-pinion)</t>
-  </si>
-  <si>
-    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, Table III (thông số ma sát bánh răng dùng trong mô phỏng Simulink của chính bài báo)</t>
-  </si>
-  <si>
     <t>c</t>
   </si>
   <si>
     <t>không thứ nguyên</t>
   </si>
   <si>
-    <t>Hệ số làm mịn hàm tanh(c*theta_dot) thay cho sign(theta_dot) - chống rung giật (chattering) số khi giải ODE qua theta_dot=0</t>
-  </si>
-  <si>
-    <t>Tự chọn (lựa chọn số học để ổn định số, không phải đại lượng đo được/trích dẫn)</t>
-  </si>
-  <si>
     <t>m</t>
   </si>
   <si>
@@ -218,6 +185,63 @@
   </si>
   <si>
     <t>CG - cầu sau (CÙNG giá trị/nguồn với l_r ở sheet Cum2, không định nghĩa lại)</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>N.m/rad</t>
+  </si>
+  <si>
+    <t>Do cung thanh xoan noi vo-lang (J1) va cot lai+motor+rack quy doi (J2)</t>
+  </si>
+  <si>
+    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, PT(14), do thuc nghiem tren xe Hyundai i30 bang nhan dang he thong (system identification, kich thich sin quet tan so, khop Bode plot)</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, PT(14)</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>T_f</t>
+  </si>
+  <si>
+    <t>Mo-men ma sat kho Coulomb giua cac cap banh rang (motor-cot lai, thuoc lai-pinion), dat o phuong trinh J2</t>
+  </si>
+  <si>
+    <t>[1] Lee, Kim, Kim (2018), IEEE TCST, Table III (thong so ma sat banh rang dung trong mo phong Simulink cua chinh bai bao)</t>
+  </si>
+  <si>
+    <t>khong thu nguyen</t>
+  </si>
+  <si>
+    <t>He so lam min ham tanh(c*theta2_dot) thay cho sign(theta2_dot) - chong rung giat (chattering) so khi giai ODE qua theta2_dot=0</t>
+  </si>
+  <si>
+    <t>Tu chon (lua chon so hoc de on dinh so, khong phai dai luong do duoc/trich dan)</t>
+  </si>
+  <si>
+    <t>He so can (damping) phia vo-lang (J1). Luu y thuat ngu: [1] goi la 'damping coefficient', KHONG goi la friction - tach biet han voi ma sat kho T_f</t>
+  </si>
+  <si>
+    <t>He so can (damping) phia J2 (cot lai+motor+rack quy doi). Cung thuat ngu voi C1 - xem ghi chu o dong C1</t>
+  </si>
+  <si>
+    <t>Quan tinh vo-lang (phia tai xe)</t>
+  </si>
+  <si>
+    <t>Quan tinh cot lai + motor tro luc (qua ty so truyen) + thanh rang/pinion (qua ban kinh pinion), quy doi ve truc theta2</t>
   </si>
 </sst>
 </file>
@@ -261,9 +285,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -279,6 +309,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -598,14 +632,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE1C4242-A034-41E0-8A93-F79CD5EB610C}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" customWidth="1"/>
     <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="131.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="126.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="70.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -618,79 +652,130 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B2">
-        <v>0.154</v>
+        <v>143.24</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
+        <v>49</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="B3">
-        <v>1.6</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="B4">
+        <v>0.25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5">
+        <v>0.11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6">
+        <v>1.35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5">
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
         <v>100</v>
       </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
-        <v>20</v>
+      <c r="C8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -729,172 +814,172 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>1573</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>1.1000000000000001</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>1.58</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>9.81</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>80000</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B7">
         <v>80000</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B8">
         <v>1.3</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B9">
         <v>-1</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="B10">
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B11">
         <v>4.8000000000000001E-2</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -933,70 +1018,70 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>1573</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B3">
         <v>2873</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>1.1000000000000001</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B5">
         <v>1.58</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>